<commit_message>
01 mais rápido, inventário revisto e ajustes do relatório
- 01: enxugar_pnadc() antes de derivar e cache dos subsets nos testes
  (preparar_design_teste()) — 47,4 -> 38,5 min, memória pedida 15,2 -> 10,0 GB;
  as 14 saídas saem idênticas byte a byte
- 09/modelo: dimensão "qualidade" -> "insercao" ("Inserção no mercado de
  trabalho"); Proporcao_Populacao_14_59 entra na Tabela 7 (base: população total)
- CONTEXTO §4: inventário de scripts revisto (faltavam 01a, 10, 10b, 11, 12, 13
  e os módulos); CLAUDE.md sem a nota de tabela desatualizada
</commit_message>
<xml_diff>
--- a/output/variaveis_indicadores.xlsx
+++ b/output/variaveis_indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matheus.barbosa\Desktop\Repositorios\PNADC-Piaui-desagregada\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9DCED9-838B-40B6-A245-806FE6BDF43C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D6A3BE3-1AF9-4B4F-A4C3-D8D6E8093F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="495" yWindow="1635" windowWidth="27810" windowHeight="12345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12945" yWindow="4095" windowWidth="27810" windowHeight="12345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicadores" sheetId="1" r:id="rId1"/>
@@ -58,9 +58,6 @@
     <t>Total (pessoas)</t>
   </si>
   <si>
-    <t>Qualidade da ocupação</t>
-  </si>
-  <si>
     <t>Rendimento e desigualdade</t>
   </si>
   <si>
@@ -266,6 +263,9 @@
   </si>
   <si>
     <t>Pessoas que não estavam trabalhando mas dispostas a trabalhar e procuraram emprego na semana de referência</t>
+  </si>
+  <si>
+    <t>Inserção no mercado de trabalho</t>
   </si>
 </sst>
 </file>
@@ -354,10 +354,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -721,388 +721,388 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="33.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4" t="s">
+    </row>
+    <row r="19" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="6"/>
+      <c r="B24" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="6"/>
+      <c r="B25" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="6"/>
+      <c r="B28" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="33.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D23" s="6" t="s">
+      <c r="C28" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D31" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="4"/>
-      <c r="B24" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
-      <c r="B25" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="4"/>
-      <c r="B28" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B8:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="A2:A13"/>
+    <mergeCell ref="A14:A20"/>
+    <mergeCell ref="A21:A25"/>
+    <mergeCell ref="A26:A30"/>
+    <mergeCell ref="A31:A34"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="B31:B34"/>
     <mergeCell ref="B26:B27"/>
     <mergeCell ref="B29:B30"/>
-    <mergeCell ref="A2:A13"/>
-    <mergeCell ref="A14:A20"/>
-    <mergeCell ref="A21:A25"/>
-    <mergeCell ref="A26:A30"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B8:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="B16:B17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>